<commit_message>
added interactive plot and fixed penalties
</commit_message>
<xml_diff>
--- a/datasets/sofascore/leagueStats/leagueStats_test.xlsx
+++ b/datasets/sofascore/leagueStats/leagueStats_test.xlsx
@@ -1037,10 +1037,10 @@
         <v>1.322996933051945</v>
       </c>
       <c r="H12" t="n">
-        <v>1.779999971389771</v>
+        <v>1.659999966621399</v>
       </c>
       <c r="I12" t="n">
-        <v>0.800000011920929</v>
+        <v>0.6899999976158142</v>
       </c>
       <c r="J12" t="n">
         <v>1</v>
@@ -1049,13 +1049,13 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>1.54</v>
+        <v>1.65</v>
       </c>
       <c r="M12" t="n">
-        <v>0.52</v>
+        <v>0.63</v>
       </c>
       <c r="N12" t="n">
-        <v>2.06</v>
+        <v>2.29</v>
       </c>
       <c r="O12" t="n">
         <v>4</v>
@@ -1448,7 +1448,7 @@
         <v>2.240000009536743</v>
       </c>
       <c r="I20" t="n">
-        <v>0.5899999737739563</v>
+        <v>0.4799999892711639</v>
       </c>
       <c r="J20" t="n">
         <v>1</v>
@@ -1460,10 +1460,10 @@
         <v>0.27</v>
       </c>
       <c r="M20" t="n">
-        <v>0.62</v>
+        <v>0.73</v>
       </c>
       <c r="N20" t="n">
-        <v>0.89</v>
+        <v>1</v>
       </c>
       <c r="O20" t="n">
         <v>2</v>
@@ -1652,7 +1652,7 @@
         <v>2.299999952316284</v>
       </c>
       <c r="I24" t="n">
-        <v>2.259999990463257</v>
+        <v>2.150000095367432</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1664,10 +1664,10 @@
         <v>0.65</v>
       </c>
       <c r="M24" t="n">
-        <v>1.08</v>
+        <v>1.19</v>
       </c>
       <c r="N24" t="n">
-        <v>1.73</v>
+        <v>1.84</v>
       </c>
       <c r="O24" t="n">
         <v>3</v>
@@ -2060,7 +2060,7 @@
         <v>0.7699999809265137</v>
       </c>
       <c r="I32" t="n">
-        <v>1.299999952316284</v>
+        <v>1.190000057220459</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -2072,10 +2072,10 @@
         <v>0.22</v>
       </c>
       <c r="M32" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.05</v>
       </c>
       <c r="N32" t="n">
-        <v>1.16</v>
+        <v>1.27</v>
       </c>
       <c r="O32" t="n">
         <v>3</v>
@@ -2108,7 +2108,7 @@
         <v>0.5463900938630171</v>
       </c>
       <c r="H33" t="n">
-        <v>1.230000019073486</v>
+        <v>1.120000004768372</v>
       </c>
       <c r="I33" t="n">
         <v>0.7200000286102295</v>
@@ -2120,13 +2120,13 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>0.36</v>
+        <v>0.47</v>
       </c>
       <c r="M33" t="n">
         <v>0.17</v>
       </c>
       <c r="N33" t="n">
-        <v>0.53</v>
+        <v>0.64</v>
       </c>
       <c r="O33" t="n">
         <v>3</v>
@@ -2159,7 +2159,7 @@
         <v>0.469316408038134</v>
       </c>
       <c r="H34" t="n">
-        <v>0.8199999928474426</v>
+        <v>0.7099999785423279</v>
       </c>
       <c r="I34" t="n">
         <v>0.6299999952316284</v>
@@ -2171,13 +2171,13 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>0.72</v>
+        <v>0.83</v>
       </c>
       <c r="M34" t="n">
         <v>0.16</v>
       </c>
       <c r="N34" t="n">
-        <v>0.88</v>
+        <v>0.99</v>
       </c>
       <c r="O34" t="n">
         <v>2</v>
@@ -2363,7 +2363,7 @@
         <v>1.662507569417363</v>
       </c>
       <c r="H38" t="n">
-        <v>0.8100000023841858</v>
+        <v>0.699999988079071</v>
       </c>
       <c r="I38" t="n">
         <v>1.409999966621399</v>
@@ -2375,13 +2375,13 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>0.55</v>
+        <v>0.66</v>
       </c>
       <c r="M38" t="n">
         <v>0.25</v>
       </c>
       <c r="N38" t="n">
-        <v>0.8</v>
+        <v>0.91</v>
       </c>
       <c r="O38" t="n">
         <v>3</v>
@@ -2519,7 +2519,7 @@
         <v>1.799999952316284</v>
       </c>
       <c r="I41" t="n">
-        <v>1.679999947547913</v>
+        <v>1.570000052452087</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -2531,10 +2531,10 @@
         <v>0.72</v>
       </c>
       <c r="M41" t="n">
-        <v>0.98</v>
+        <v>1.09</v>
       </c>
       <c r="N41" t="n">
-        <v>1.7</v>
+        <v>1.81</v>
       </c>
       <c r="O41" t="n">
         <v>5</v>
@@ -2876,7 +2876,7 @@
         <v>1.460000038146973</v>
       </c>
       <c r="I48" t="n">
-        <v>0.9200000166893005</v>
+        <v>0.8100000023841858</v>
       </c>
       <c r="J48" t="n">
         <v>1</v>
@@ -2888,10 +2888,10 @@
         <v>0.35</v>
       </c>
       <c r="M48" t="n">
-        <v>0.45</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="N48" t="n">
-        <v>0.8</v>
+        <v>0.91</v>
       </c>
       <c r="O48" t="n">
         <v>3</v>
@@ -2927,7 +2927,7 @@
         <v>0.7300000190734863</v>
       </c>
       <c r="I49" t="n">
-        <v>2.200000047683716</v>
+        <v>2.079999923706055</v>
       </c>
       <c r="J49" t="n">
         <v>0</v>
@@ -2939,10 +2939,10 @@
         <v>0.02</v>
       </c>
       <c r="M49" t="n">
-        <v>0.76</v>
+        <v>0.87</v>
       </c>
       <c r="N49" t="n">
-        <v>0.78</v>
+        <v>0.89</v>
       </c>
       <c r="O49" t="n">
         <v>3</v>
@@ -2975,7 +2975,7 @@
         <v>0.7615197636187041</v>
       </c>
       <c r="H50" t="n">
-        <v>0.800000011920929</v>
+        <v>0.6899999976158142</v>
       </c>
       <c r="I50" t="n">
         <v>1.110000014305115</v>
@@ -2987,13 +2987,13 @@
         <v>0</v>
       </c>
       <c r="L50" t="n">
-        <v>0.5</v>
+        <v>0.61</v>
       </c>
       <c r="M50" t="n">
         <v>0.35</v>
       </c>
       <c r="N50" t="n">
-        <v>0.85</v>
+        <v>0.96</v>
       </c>
       <c r="O50" t="n">
         <v>3</v>
@@ -3080,7 +3080,7 @@
         <v>1.269999980926514</v>
       </c>
       <c r="I52" t="n">
-        <v>1.409999966621399</v>
+        <v>1.299999952316284</v>
       </c>
       <c r="J52" t="n">
         <v>0</v>
@@ -3092,10 +3092,10 @@
         <v>0.48</v>
       </c>
       <c r="M52" t="n">
-        <v>0.97</v>
+        <v>1.08</v>
       </c>
       <c r="N52" t="n">
-        <v>1.45</v>
+        <v>1.56</v>
       </c>
       <c r="O52" t="n">
         <v>0</v>
@@ -3128,7 +3128,7 @@
         <v>1.778500117361556</v>
       </c>
       <c r="H53" t="n">
-        <v>0.6800000071525574</v>
+        <v>0.5699999928474426</v>
       </c>
       <c r="I53" t="n">
         <v>1.570000052452087</v>
@@ -3140,13 +3140,13 @@
         <v>0</v>
       </c>
       <c r="L53" t="n">
-        <v>0.58</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="M53" t="n">
         <v>0.21</v>
       </c>
       <c r="N53" t="n">
-        <v>0.78</v>
+        <v>0.89</v>
       </c>
       <c r="O53" t="n">
         <v>6</v>
@@ -3539,7 +3539,7 @@
         <v>0.9900000095367432</v>
       </c>
       <c r="I61" t="n">
-        <v>1.350000023841858</v>
+        <v>1.240000009536743</v>
       </c>
       <c r="J61" t="n">
         <v>0</v>
@@ -3551,10 +3551,10 @@
         <v>0.14</v>
       </c>
       <c r="M61" t="n">
-        <v>0.41</v>
+        <v>0.52</v>
       </c>
       <c r="N61" t="n">
-        <v>0.55</v>
+        <v>0.66</v>
       </c>
       <c r="O61" t="n">
         <v>0</v>
@@ -3893,7 +3893,7 @@
         <v>0.025717673823237</v>
       </c>
       <c r="H68" t="n">
-        <v>1.559999942779541</v>
+        <v>1.450000047683716</v>
       </c>
       <c r="I68" t="n">
         <v>0.05000000074505806</v>
@@ -3905,13 +3905,13 @@
         <v>0</v>
       </c>
       <c r="L68" t="n">
-        <v>0.64</v>
+        <v>0.75</v>
       </c>
       <c r="M68" t="n">
         <v>0.03</v>
       </c>
       <c r="N68" t="n">
-        <v>0.67</v>
+        <v>0.78</v>
       </c>
       <c r="O68" t="n">
         <v>0</v>
@@ -3995,7 +3995,7 @@
         <v>1.141721876338126</v>
       </c>
       <c r="H70" t="n">
-        <v>1.360000014305115</v>
+        <v>1.25</v>
       </c>
       <c r="I70" t="n">
         <v>0.9800000190734863</v>
@@ -4007,13 +4007,13 @@
         <v>1</v>
       </c>
       <c r="L70" t="n">
-        <v>0.62</v>
+        <v>0.73</v>
       </c>
       <c r="M70" t="n">
         <v>0.16</v>
       </c>
       <c r="N70" t="n">
-        <v>0.77</v>
+        <v>0.88</v>
       </c>
       <c r="O70" t="n">
         <v>2</v>
@@ -4100,7 +4100,7 @@
         <v>1.870000004768372</v>
       </c>
       <c r="I72" t="n">
-        <v>0.4399999976158142</v>
+        <v>0.3300000131130219</v>
       </c>
       <c r="J72" t="n">
         <v>0</v>
@@ -4112,10 +4112,10 @@
         <v>0.33</v>
       </c>
       <c r="M72" t="n">
-        <v>1.07</v>
+        <v>1.18</v>
       </c>
       <c r="N72" t="n">
-        <v>1.4</v>
+        <v>1.51</v>
       </c>
       <c r="O72" t="n">
         <v>4</v>
@@ -4250,10 +4250,10 @@
         <v>1.905408421570068</v>
       </c>
       <c r="H75" t="n">
-        <v>0.6200000047683716</v>
+        <v>0.5099999904632568</v>
       </c>
       <c r="I75" t="n">
-        <v>1.289999961853027</v>
+        <v>1.179999947547913</v>
       </c>
       <c r="J75" t="n">
         <v>0</v>
@@ -4262,13 +4262,13 @@
         <v>0</v>
       </c>
       <c r="L75" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="M75" t="n">
         <v>0.72</v>
       </c>
-      <c r="M75" t="n">
-        <v>0.61</v>
-      </c>
       <c r="N75" t="n">
-        <v>1.33</v>
+        <v>1.55</v>
       </c>
       <c r="O75" t="n">
         <v>4</v>
@@ -4505,7 +4505,7 @@
         <v>1.018078027293079</v>
       </c>
       <c r="H80" t="n">
-        <v>2.230000019073486</v>
+        <v>2.059999942779541</v>
       </c>
       <c r="I80" t="n">
         <v>0.75</v>
@@ -4517,13 +4517,13 @@
         <v>0</v>
       </c>
       <c r="L80" t="n">
-        <v>1.51</v>
+        <v>1.69</v>
       </c>
       <c r="M80" t="n">
         <v>0.26</v>
       </c>
       <c r="N80" t="n">
-        <v>1.78</v>
+        <v>1.95</v>
       </c>
       <c r="O80" t="n">
         <v>4</v>
@@ -4607,7 +4607,7 @@
         <v>0.8294987287372341</v>
       </c>
       <c r="H82" t="n">
-        <v>0.4799999892711639</v>
+        <v>0.3700000047683716</v>
       </c>
       <c r="I82" t="n">
         <v>1.120000004768372</v>
@@ -4619,13 +4619,13 @@
         <v>0</v>
       </c>
       <c r="L82" t="n">
-        <v>0.68</v>
+        <v>0.79</v>
       </c>
       <c r="M82" t="n">
         <v>0.29</v>
       </c>
       <c r="N82" t="n">
-        <v>0.97</v>
+        <v>1.08</v>
       </c>
       <c r="O82" t="n">
         <v>1</v>
@@ -4811,7 +4811,7 @@
         <v>0.534137243404987</v>
       </c>
       <c r="H86" t="n">
-        <v>2.259999990463257</v>
+        <v>2.089999914169312</v>
       </c>
       <c r="I86" t="n">
         <v>0.7599999904632568</v>
@@ -4823,13 +4823,13 @@
         <v>0</v>
       </c>
       <c r="L86" t="n">
-        <v>0.9</v>
+        <v>1.07</v>
       </c>
       <c r="M86" t="n">
         <v>0.22</v>
       </c>
       <c r="N86" t="n">
-        <v>1.12</v>
+        <v>1.3</v>
       </c>
       <c r="O86" t="n">
         <v>4</v>
@@ -4964,7 +4964,7 @@
         <v>0.692326349206269</v>
       </c>
       <c r="H89" t="n">
-        <v>2.369999885559082</v>
+        <v>2.259999990463257</v>
       </c>
       <c r="I89" t="n">
         <v>1.059999942779541</v>
@@ -4976,13 +4976,13 @@
         <v>0</v>
       </c>
       <c r="L89" t="n">
-        <v>0.26</v>
+        <v>0.37</v>
       </c>
       <c r="M89" t="n">
         <v>0.37</v>
       </c>
       <c r="N89" t="n">
-        <v>0.63</v>
+        <v>0.74</v>
       </c>
       <c r="O89" t="n">
         <v>3</v>
@@ -5171,7 +5171,7 @@
         <v>0.7400000095367432</v>
       </c>
       <c r="I93" t="n">
-        <v>0.6100000143051147</v>
+        <v>0.5</v>
       </c>
       <c r="J93" t="n">
         <v>0</v>
@@ -5183,10 +5183,10 @@
         <v>0.14</v>
       </c>
       <c r="M93" t="n">
-        <v>0.63</v>
+        <v>0.75</v>
       </c>
       <c r="N93" t="n">
-        <v>0.78</v>
+        <v>0.89</v>
       </c>
       <c r="O93" t="n">
         <v>0</v>
@@ -5375,7 +5375,7 @@
         <v>1.620000004768372</v>
       </c>
       <c r="I97" t="n">
-        <v>1.120000004768372</v>
+        <v>1.009999990463257</v>
       </c>
       <c r="J97" t="n">
         <v>0</v>
@@ -5387,10 +5387,10 @@
         <v>0.7</v>
       </c>
       <c r="M97" t="n">
-        <v>0.4</v>
+        <v>0.51</v>
       </c>
       <c r="N97" t="n">
-        <v>1.1</v>
+        <v>1.21</v>
       </c>
       <c r="O97" t="n">
         <v>4</v>
@@ -5477,7 +5477,7 @@
         <v>2.900000095367432</v>
       </c>
       <c r="I99" t="n">
-        <v>1.679999947547913</v>
+        <v>1.559999942779541</v>
       </c>
       <c r="J99" t="n">
         <v>1</v>
@@ -5489,10 +5489,10 @@
         <v>0.86</v>
       </c>
       <c r="M99" t="n">
-        <v>0.27</v>
+        <v>0.38</v>
       </c>
       <c r="N99" t="n">
-        <v>1.13</v>
+        <v>1.24</v>
       </c>
       <c r="O99" t="n">
         <v>0</v>
@@ -5834,7 +5834,7 @@
         <v>1.470000028610229</v>
       </c>
       <c r="I106" t="n">
-        <v>1.009999990463257</v>
+        <v>0.8999999761581421</v>
       </c>
       <c r="J106" t="n">
         <v>0</v>
@@ -5846,10 +5846,10 @@
         <v>0.42</v>
       </c>
       <c r="M106" t="n">
-        <v>1.06</v>
+        <v>1.17</v>
       </c>
       <c r="N106" t="n">
-        <v>1.47</v>
+        <v>1.58</v>
       </c>
       <c r="O106" t="n">
         <v>4</v>
@@ -5885,7 +5885,7 @@
         <v>1.340000033378601</v>
       </c>
       <c r="I107" t="n">
-        <v>0.949999988079071</v>
+        <v>0.8299999833106995</v>
       </c>
       <c r="J107" t="n">
         <v>0</v>
@@ -5897,10 +5897,10 @@
         <v>0.43</v>
       </c>
       <c r="M107" t="n">
-        <v>1.08</v>
+        <v>1.19</v>
       </c>
       <c r="N107" t="n">
-        <v>1.51</v>
+        <v>1.62</v>
       </c>
       <c r="O107" t="n">
         <v>3</v>
@@ -5984,10 +5984,10 @@
         <v>1.651833647900813</v>
       </c>
       <c r="H109" t="n">
-        <v>1.129999995231628</v>
+        <v>1.009999990463257</v>
       </c>
       <c r="I109" t="n">
-        <v>0.6800000071525574</v>
+        <v>0.5699999928474426</v>
       </c>
       <c r="J109" t="n">
         <v>0</v>
@@ -5996,13 +5996,13 @@
         <v>0</v>
       </c>
       <c r="L109" t="n">
-        <v>0.46</v>
+        <v>0.57</v>
       </c>
       <c r="M109" t="n">
-        <v>0.97</v>
+        <v>1.08</v>
       </c>
       <c r="N109" t="n">
-        <v>1.43</v>
+        <v>1.65</v>
       </c>
       <c r="O109" t="n">
         <v>4</v>
@@ -6035,7 +6035,7 @@
         <v>1.057036051061005</v>
       </c>
       <c r="H110" t="n">
-        <v>1.340000033378601</v>
+        <v>1.230000019073486</v>
       </c>
       <c r="I110" t="n">
         <v>1.090000033378601</v>
@@ -6047,13 +6047,13 @@
         <v>0</v>
       </c>
       <c r="L110" t="n">
-        <v>0.19</v>
+        <v>0.3</v>
       </c>
       <c r="M110" t="n">
         <v>0.03</v>
       </c>
       <c r="N110" t="n">
-        <v>0.22</v>
+        <v>0.33</v>
       </c>
       <c r="O110" t="n">
         <v>2</v>
@@ -6191,7 +6191,7 @@
         <v>1.429999947547913</v>
       </c>
       <c r="I113" t="n">
-        <v>1.419999957084656</v>
+        <v>1.309999942779541</v>
       </c>
       <c r="J113" t="n">
         <v>0</v>
@@ -6203,10 +6203,10 @@
         <v>0.02</v>
       </c>
       <c r="M113" t="n">
-        <v>0.92</v>
+        <v>1.03</v>
       </c>
       <c r="N113" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.05</v>
       </c>
       <c r="O113" t="n">
         <v>3</v>
@@ -6494,7 +6494,7 @@
         <v>1.063483301550145</v>
       </c>
       <c r="H119" t="n">
-        <v>1.570000052452087</v>
+        <v>1.460000038146973</v>
       </c>
       <c r="I119" t="n">
         <v>0.6399999856948853</v>
@@ -6506,13 +6506,13 @@
         <v>0</v>
       </c>
       <c r="L119" t="n">
-        <v>0.35</v>
+        <v>0.46</v>
       </c>
       <c r="M119" t="n">
         <v>0.42</v>
       </c>
       <c r="N119" t="n">
-        <v>0.77</v>
+        <v>0.88</v>
       </c>
       <c r="O119" t="n">
         <v>1</v>
@@ -6545,7 +6545,7 @@
         <v>2.806447237730022</v>
       </c>
       <c r="H120" t="n">
-        <v>0.949999988079071</v>
+        <v>0.8399999737739563</v>
       </c>
       <c r="I120" t="n">
         <v>2.029999971389771</v>
@@ -6557,13 +6557,13 @@
         <v>0</v>
       </c>
       <c r="L120" t="n">
-        <v>0.55</v>
+        <v>0.66</v>
       </c>
       <c r="M120" t="n">
         <v>0.78</v>
       </c>
       <c r="N120" t="n">
-        <v>1.33</v>
+        <v>1.44</v>
       </c>
       <c r="O120" t="n">
         <v>6</v>
@@ -6599,7 +6599,7 @@
         <v>2.119999885559082</v>
       </c>
       <c r="I121" t="n">
-        <v>0.8999999761581421</v>
+        <v>0.7900000214576721</v>
       </c>
       <c r="J121" t="n">
         <v>0</v>
@@ -6611,10 +6611,10 @@
         <v>0.36</v>
       </c>
       <c r="M121" t="n">
-        <v>0.64</v>
+        <v>0.76</v>
       </c>
       <c r="N121" t="n">
-        <v>1.01</v>
+        <v>1.12</v>
       </c>
       <c r="O121" t="n">
         <v>4</v>
@@ -6752,7 +6752,7 @@
         <v>1.039999961853027</v>
       </c>
       <c r="I124" t="n">
-        <v>0.8799999952316284</v>
+        <v>0.7599999904632568</v>
       </c>
       <c r="J124" t="n">
         <v>0</v>
@@ -6764,10 +6764,10 @@
         <v>0.08</v>
       </c>
       <c r="M124" t="n">
-        <v>0.71</v>
+        <v>0.82</v>
       </c>
       <c r="N124" t="n">
-        <v>0.79</v>
+        <v>0.9</v>
       </c>
       <c r="O124" t="n">
         <v>2</v>
@@ -6905,7 +6905,7 @@
         <v>0.7300000190734863</v>
       </c>
       <c r="I127" t="n">
-        <v>1.080000042915344</v>
+        <v>0.9700000286102295</v>
       </c>
       <c r="J127" t="n">
         <v>0</v>
@@ -6917,10 +6917,10 @@
         <v>0.27</v>
       </c>
       <c r="M127" t="n">
-        <v>0.66</v>
+        <v>0.77</v>
       </c>
       <c r="N127" t="n">
-        <v>0.93</v>
+        <v>1.04</v>
       </c>
       <c r="O127" t="n">
         <v>3</v>
@@ -7106,7 +7106,7 @@
         <v>2.133399207144965</v>
       </c>
       <c r="H131" t="n">
-        <v>2.650000095367432</v>
+        <v>2.539999961853027</v>
       </c>
       <c r="I131" t="n">
         <v>1.419999957084656</v>
@@ -7118,13 +7118,13 @@
         <v>0</v>
       </c>
       <c r="L131" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.18</v>
       </c>
       <c r="M131" t="n">
         <v>0.71</v>
       </c>
       <c r="N131" t="n">
-        <v>0.78</v>
+        <v>0.89</v>
       </c>
       <c r="O131" t="n">
         <v>4</v>
@@ -7160,7 +7160,7 @@
         <v>1.25</v>
       </c>
       <c r="I132" t="n">
-        <v>0.699999988079071</v>
+        <v>0.5899999737739563</v>
       </c>
       <c r="J132" t="n">
         <v>0</v>
@@ -7172,10 +7172,10 @@
         <v>0.25</v>
       </c>
       <c r="M132" t="n">
-        <v>0.53</v>
+        <v>0.64</v>
       </c>
       <c r="N132" t="n">
-        <v>0.77</v>
+        <v>0.88</v>
       </c>
       <c r="O132" t="n">
         <v>4</v>
@@ -7262,7 +7262,7 @@
         <v>1.25</v>
       </c>
       <c r="I134" t="n">
-        <v>1.059999942779541</v>
+        <v>0.949999988079071</v>
       </c>
       <c r="J134" t="n">
         <v>0</v>
@@ -7274,10 +7274,10 @@
         <v>0.26</v>
       </c>
       <c r="M134" t="n">
-        <v>0.52</v>
+        <v>0.63</v>
       </c>
       <c r="N134" t="n">
-        <v>0.78</v>
+        <v>0.89</v>
       </c>
       <c r="O134" t="n">
         <v>4</v>
@@ -7310,7 +7310,7 @@
         <v>0.9137102840468209</v>
       </c>
       <c r="H135" t="n">
-        <v>1.289999961853027</v>
+        <v>1.179999947547913</v>
       </c>
       <c r="I135" t="n">
         <v>1.080000042915344</v>
@@ -7322,13 +7322,13 @@
         <v>0</v>
       </c>
       <c r="L135" t="n">
-        <v>0.79</v>
+        <v>0.9</v>
       </c>
       <c r="M135" t="n">
         <v>0.17</v>
       </c>
       <c r="N135" t="n">
-        <v>0.95</v>
+        <v>1.06</v>
       </c>
       <c r="O135" t="n">
         <v>2</v>
@@ -7517,7 +7517,7 @@
         <v>1.799999952316284</v>
       </c>
       <c r="I139" t="n">
-        <v>0.5600000023841858</v>
+        <v>0.449999988079071</v>
       </c>
       <c r="J139" t="n">
         <v>0</v>
@@ -7529,10 +7529,10 @@
         <v>0.28</v>
       </c>
       <c r="M139" t="n">
-        <v>0.68</v>
+        <v>0.79</v>
       </c>
       <c r="N139" t="n">
-        <v>0.96</v>
+        <v>1.07</v>
       </c>
       <c r="O139" t="n">
         <v>1</v>
@@ -7568,7 +7568,7 @@
         <v>1.480000019073486</v>
       </c>
       <c r="I140" t="n">
-        <v>0.8700000047683716</v>
+        <v>0.7599999904632568</v>
       </c>
       <c r="J140" t="n">
         <v>0</v>
@@ -7580,10 +7580,10 @@
         <v>0.31</v>
       </c>
       <c r="M140" t="n">
-        <v>0.72</v>
+        <v>0.84</v>
       </c>
       <c r="N140" t="n">
-        <v>1.04</v>
+        <v>1.15</v>
       </c>
       <c r="O140" t="n">
         <v>3</v>
@@ -7616,7 +7616,7 @@
         <v>1.695289418101309</v>
       </c>
       <c r="H141" t="n">
-        <v>0.4399999976158142</v>
+        <v>0.3300000131130219</v>
       </c>
       <c r="I141" t="n">
         <v>1.970000028610229</v>
@@ -7628,13 +7628,13 @@
         <v>0</v>
       </c>
       <c r="L141" t="n">
-        <v>0.58</v>
+        <v>0.7</v>
       </c>
       <c r="M141" t="n">
         <v>0.27</v>
       </c>
       <c r="N141" t="n">
-        <v>0.85</v>
+        <v>0.97</v>
       </c>
       <c r="O141" t="n">
         <v>5</v>
@@ -8282,7 +8282,7 @@
         <v>1.379999995231628</v>
       </c>
       <c r="I154" t="n">
-        <v>1.620000004768372</v>
+        <v>1.509999990463257</v>
       </c>
       <c r="J154" t="n">
         <v>0</v>
@@ -8294,10 +8294,10 @@
         <v>0.05</v>
       </c>
       <c r="M154" t="n">
-        <v>0.92</v>
+        <v>1.03</v>
       </c>
       <c r="N154" t="n">
-        <v>0.97</v>
+        <v>1.08</v>
       </c>
       <c r="O154" t="n">
         <v>4</v>
@@ -8333,7 +8333,7 @@
         <v>0.5</v>
       </c>
       <c r="I155" t="n">
-        <v>0.8500000238418579</v>
+        <v>0.7400000095367432</v>
       </c>
       <c r="J155" t="n">
         <v>0</v>
@@ -8345,10 +8345,10 @@
         <v>0.08</v>
       </c>
       <c r="M155" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="N155" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.06</v>
       </c>
       <c r="O155" t="n">
         <v>1</v>
@@ -8639,7 +8639,7 @@
         <v>1.700000047683716</v>
       </c>
       <c r="I161" t="n">
-        <v>0.6299999952316284</v>
+        <v>0.5199999809265137</v>
       </c>
       <c r="J161" t="n">
         <v>0</v>
@@ -8651,10 +8651,10 @@
         <v>0.16</v>
       </c>
       <c r="M161" t="n">
-        <v>0.64</v>
+        <v>0.75</v>
       </c>
       <c r="N161" t="n">
-        <v>0.8</v>
+        <v>0.91</v>
       </c>
       <c r="O161" t="n">
         <v>4</v>
@@ -8942,7 +8942,7 @@
         <v>0.393704540096223</v>
       </c>
       <c r="H167" t="n">
-        <v>1.440000057220459</v>
+        <v>1.330000042915344</v>
       </c>
       <c r="I167" t="n">
         <v>0.4900000095367432</v>
@@ -8954,13 +8954,13 @@
         <v>0</v>
       </c>
       <c r="L167" t="n">
-        <v>1.03</v>
+        <v>1.14</v>
       </c>
       <c r="M167" t="n">
         <v>0.1</v>
       </c>
       <c r="N167" t="n">
-        <v>1.13</v>
+        <v>1.24</v>
       </c>
       <c r="O167" t="n">
         <v>2</v>
@@ -9248,7 +9248,7 @@
         <v>0.590074462816124</v>
       </c>
       <c r="H173" t="n">
-        <v>1.450000047683716</v>
+        <v>1.340000033378601</v>
       </c>
       <c r="I173" t="n">
         <v>0.2300000041723251</v>
@@ -9260,13 +9260,13 @@
         <v>0</v>
       </c>
       <c r="L173" t="n">
-        <v>0.79</v>
+        <v>0.9</v>
       </c>
       <c r="M173" t="n">
         <v>0.36</v>
       </c>
       <c r="N173" t="n">
-        <v>1.14</v>
+        <v>1.25</v>
       </c>
       <c r="O173" t="n">
         <v>1</v>
@@ -9401,7 +9401,7 @@
         <v>0.284416534006598</v>
       </c>
       <c r="H176" t="n">
-        <v>2.480000019073486</v>
+        <v>2.369999885559082</v>
       </c>
       <c r="I176" t="n">
         <v>0.2599999904632568</v>
@@ -9413,13 +9413,13 @@
         <v>0</v>
       </c>
       <c r="L176" t="n">
-        <v>0.29</v>
+        <v>0.41</v>
       </c>
       <c r="M176" t="n">
         <v>0.02</v>
       </c>
       <c r="N176" t="n">
-        <v>0.32</v>
+        <v>0.43</v>
       </c>
       <c r="O176" t="n">
         <v>2</v>
@@ -9707,10 +9707,10 @@
         <v>1.670245617666837</v>
       </c>
       <c r="H182" t="n">
-        <v>0.800000011920929</v>
+        <v>0.6899999976158142</v>
       </c>
       <c r="I182" t="n">
-        <v>1.279999971389771</v>
+        <v>1.159999966621399</v>
       </c>
       <c r="J182" t="n">
         <v>0</v>
@@ -9719,13 +9719,13 @@
         <v>0</v>
       </c>
       <c r="L182" t="n">
-        <v>0.77</v>
+        <v>0.88</v>
       </c>
       <c r="M182" t="n">
-        <v>0.4</v>
+        <v>0.51</v>
       </c>
       <c r="N182" t="n">
-        <v>1.17</v>
+        <v>1.39</v>
       </c>
       <c r="O182" t="n">
         <v>3</v>
@@ -9914,7 +9914,7 @@
         <v>1.5</v>
       </c>
       <c r="I186" t="n">
-        <v>1.129999995231628</v>
+        <v>1.019999980926514</v>
       </c>
       <c r="J186" t="n">
         <v>0</v>
@@ -9926,10 +9926,10 @@
         <v>0.28</v>
       </c>
       <c r="M186" t="n">
-        <v>0.67</v>
+        <v>0.78</v>
       </c>
       <c r="N186" t="n">
-        <v>0.95</v>
+        <v>1.06</v>
       </c>
       <c r="O186" t="n">
         <v>3</v>
@@ -9962,10 +9962,10 @@
         <v>1.719655482137201</v>
       </c>
       <c r="H187" t="n">
-        <v>1.659999966621399</v>
+        <v>1.549999952316284</v>
       </c>
       <c r="I187" t="n">
-        <v>0.9800000190734863</v>
+        <v>0.8700000047683716</v>
       </c>
       <c r="J187" t="n">
         <v>0</v>
@@ -9974,13 +9974,13 @@
         <v>0</v>
       </c>
       <c r="L187" t="n">
-        <v>1.18</v>
+        <v>1.3</v>
       </c>
       <c r="M187" t="n">
-        <v>0.74</v>
+        <v>0.85</v>
       </c>
       <c r="N187" t="n">
-        <v>1.92</v>
+        <v>2.15</v>
       </c>
       <c r="O187" t="n">
         <v>4</v>
@@ -10169,7 +10169,7 @@
         <v>3.259999990463257</v>
       </c>
       <c r="I191" t="n">
-        <v>0.6100000143051147</v>
+        <v>0.4900000095367432</v>
       </c>
       <c r="J191" t="n">
         <v>0</v>
@@ -10181,10 +10181,10 @@
         <v>0.8100000000000001</v>
       </c>
       <c r="M191" t="n">
-        <v>0.71</v>
+        <v>0.83</v>
       </c>
       <c r="N191" t="n">
-        <v>1.53</v>
+        <v>1.64</v>
       </c>
       <c r="O191" t="n">
         <v>2</v>
@@ -10268,7 +10268,7 @@
         <v>1.795822645537553</v>
       </c>
       <c r="H193" t="n">
-        <v>1.320000052452087</v>
+        <v>1.210000038146973</v>
       </c>
       <c r="I193" t="n">
         <v>1.620000004768372</v>
@@ -10280,13 +10280,13 @@
         <v>1</v>
       </c>
       <c r="L193" t="n">
-        <v>0.9</v>
+        <v>1.01</v>
       </c>
       <c r="M193" t="n">
         <v>0.18</v>
       </c>
       <c r="N193" t="n">
-        <v>1.08</v>
+        <v>1.19</v>
       </c>
       <c r="O193" t="n">
         <v>3</v>
@@ -10574,7 +10574,7 @@
         <v>0.711492316797373</v>
       </c>
       <c r="H199" t="n">
-        <v>1.059999942779541</v>
+        <v>0.9399999976158142</v>
       </c>
       <c r="I199" t="n">
         <v>0.9800000190734863</v>
@@ -10586,13 +10586,13 @@
         <v>0</v>
       </c>
       <c r="L199" t="n">
-        <v>0.39</v>
+        <v>0.5</v>
       </c>
       <c r="M199" t="n">
         <v>0.27</v>
       </c>
       <c r="N199" t="n">
-        <v>0.66</v>
+        <v>0.77</v>
       </c>
       <c r="O199" t="n">
         <v>4</v>
@@ -10676,7 +10676,7 @@
         <v>0.9358670730143841</v>
       </c>
       <c r="H201" t="n">
-        <v>1.830000042915344</v>
+        <v>1.720000028610229</v>
       </c>
       <c r="I201" t="n">
         <v>1.139999985694885</v>
@@ -10688,13 +10688,13 @@
         <v>0</v>
       </c>
       <c r="L201" t="n">
-        <v>2.26</v>
+        <v>2.37</v>
       </c>
       <c r="M201" t="n">
         <v>0.2</v>
       </c>
       <c r="N201" t="n">
-        <v>2.46</v>
+        <v>2.57</v>
       </c>
       <c r="O201" t="n">
         <v>5</v>
@@ -11189,7 +11189,7 @@
         <v>0.3899999856948853</v>
       </c>
       <c r="I211" t="n">
-        <v>1.379999995231628</v>
+        <v>1.259999990463257</v>
       </c>
       <c r="J211" t="n">
         <v>0</v>
@@ -11201,10 +11201,10 @@
         <v>0.02</v>
       </c>
       <c r="M211" t="n">
-        <v>0.93</v>
+        <v>1.04</v>
       </c>
       <c r="N211" t="n">
-        <v>0.95</v>
+        <v>1.06</v>
       </c>
       <c r="O211" t="n">
         <v>3</v>
@@ -11231,13 +11231,13 @@
         <v>2</v>
       </c>
       <c r="F212" t="n">
-        <v>5.107227601149665</v>
+        <v>5.107227601149666</v>
       </c>
       <c r="G212" t="n">
         <v>0.348652336746454</v>
       </c>
       <c r="H212" t="n">
-        <v>5.139999866485596</v>
+        <v>5.03000020980835</v>
       </c>
       <c r="I212" t="n">
         <v>0.4000000059604645</v>
@@ -11249,13 +11249,13 @@
         <v>0</v>
       </c>
       <c r="L212" t="n">
-        <v>0.04</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="M212" t="n">
         <v>0.05</v>
       </c>
       <c r="N212" t="n">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
       <c r="O212" t="n">
         <v>7</v>
@@ -11288,7 +11288,7 @@
         <v>0.515181334689255</v>
       </c>
       <c r="H213" t="n">
-        <v>1.570000052452087</v>
+        <v>1.460000038146973</v>
       </c>
       <c r="I213" t="n">
         <v>0.6800000071525574</v>
@@ -11300,13 +11300,13 @@
         <v>0</v>
       </c>
       <c r="L213" t="n">
-        <v>1.31</v>
+        <v>1.42</v>
       </c>
       <c r="M213" t="n">
         <v>0.17</v>
       </c>
       <c r="N213" t="n">
-        <v>1.47</v>
+        <v>1.58</v>
       </c>
       <c r="O213" t="n">
         <v>6</v>
@@ -11492,7 +11492,7 @@
         <v>1.654719011858103</v>
       </c>
       <c r="H217" t="n">
-        <v>3.619999885559082</v>
+        <v>3.509999990463257</v>
       </c>
       <c r="I217" t="n">
         <v>1.669999957084656</v>
@@ -11504,13 +11504,13 @@
         <v>0</v>
       </c>
       <c r="L217" t="n">
-        <v>0.63</v>
+        <v>0.74</v>
       </c>
       <c r="M217" t="n">
         <v>0.02</v>
       </c>
       <c r="N217" t="n">
-        <v>0.65</v>
+        <v>0.76</v>
       </c>
       <c r="O217" t="n">
         <v>1</v>
@@ -11645,7 +11645,7 @@
         <v>0.4451905945316</v>
       </c>
       <c r="H220" t="n">
-        <v>1.649999976158142</v>
+        <v>1.539999961853027</v>
       </c>
       <c r="I220" t="n">
         <v>0.4099999964237213</v>
@@ -11657,13 +11657,13 @@
         <v>0</v>
       </c>
       <c r="L220" t="n">
-        <v>1.08</v>
+        <v>1.19</v>
       </c>
       <c r="M220" t="n">
         <v>0.04</v>
       </c>
       <c r="N220" t="n">
-        <v>1.11</v>
+        <v>1.22</v>
       </c>
       <c r="O220" t="n">
         <v>2</v>
@@ -11747,10 +11747,10 @@
         <v>1.755172023588419</v>
       </c>
       <c r="H222" t="n">
-        <v>1.039999961853027</v>
+        <v>0.8700000047683716</v>
       </c>
       <c r="I222" t="n">
-        <v>1.440000057220459</v>
+        <v>1.330000042915344</v>
       </c>
       <c r="J222" t="n">
         <v>0</v>
@@ -11759,13 +11759,13 @@
         <v>0</v>
       </c>
       <c r="L222" t="n">
-        <v>1.08</v>
+        <v>1.25</v>
       </c>
       <c r="M222" t="n">
-        <v>0.32</v>
+        <v>0.43</v>
       </c>
       <c r="N222" t="n">
-        <v>1.4</v>
+        <v>1.68</v>
       </c>
       <c r="O222" t="n">
         <v>5</v>
@@ -12002,7 +12002,7 @@
         <v>0.6664145365357419</v>
       </c>
       <c r="H227" t="n">
-        <v>3.359999895095825</v>
+        <v>3.25</v>
       </c>
       <c r="I227" t="n">
         <v>0.7900000214576721</v>
@@ -12014,13 +12014,13 @@
         <v>0</v>
       </c>
       <c r="L227" t="n">
-        <v>1.69</v>
+        <v>1.81</v>
       </c>
       <c r="M227" t="n">
         <v>0.13</v>
       </c>
       <c r="N227" t="n">
-        <v>1.82</v>
+        <v>1.93</v>
       </c>
       <c r="O227" t="n">
         <v>1</v>
@@ -12209,7 +12209,7 @@
         <v>0.8199999928474426</v>
       </c>
       <c r="I231" t="n">
-        <v>1.440000057220459</v>
+        <v>1.330000042915344</v>
       </c>
       <c r="J231" t="n">
         <v>0</v>
@@ -12221,10 +12221,10 @@
         <v>0.37</v>
       </c>
       <c r="M231" t="n">
-        <v>1.38</v>
+        <v>1.49</v>
       </c>
       <c r="N231" t="n">
-        <v>1.75</v>
+        <v>1.86</v>
       </c>
       <c r="O231" t="n">
         <v>3</v>
@@ -12308,10 +12308,10 @@
         <v>2.560501286798734</v>
       </c>
       <c r="H233" t="n">
-        <v>0.9700000286102295</v>
+        <v>0.8600000143051147</v>
       </c>
       <c r="I233" t="n">
-        <v>1.350000023841858</v>
+        <v>1.240000009536743</v>
       </c>
       <c r="J233" t="n">
         <v>0</v>
@@ -12320,13 +12320,13 @@
         <v>0</v>
       </c>
       <c r="L233" t="n">
-        <v>0.39</v>
+        <v>0.5</v>
       </c>
       <c r="M233" t="n">
-        <v>1.21</v>
+        <v>1.32</v>
       </c>
       <c r="N233" t="n">
-        <v>1.59</v>
+        <v>1.82</v>
       </c>
       <c r="O233" t="n">
         <v>5</v>
@@ -12464,7 +12464,7 @@
         <v>1.340000033378601</v>
       </c>
       <c r="I236" t="n">
-        <v>0.3400000035762787</v>
+        <v>0.2300000041723251</v>
       </c>
       <c r="J236" t="n">
         <v>0</v>
@@ -12476,10 +12476,10 @@
         <v>0.13</v>
       </c>
       <c r="M236" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.67</v>
       </c>
       <c r="N236" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.8</v>
       </c>
       <c r="O236" t="n">
         <v>3</v>
@@ -12770,7 +12770,7 @@
         <v>0.449999988079071</v>
       </c>
       <c r="I242" t="n">
-        <v>1.259999990463257</v>
+        <v>1.149999976158142</v>
       </c>
       <c r="J242" t="n">
         <v>0</v>
@@ -12782,10 +12782,10 @@
         <v>0.32</v>
       </c>
       <c r="M242" t="n">
-        <v>1.07</v>
+        <v>1.18</v>
       </c>
       <c r="N242" t="n">
-        <v>1.39</v>
+        <v>1.5</v>
       </c>
       <c r="O242" t="n">
         <v>3</v>
@@ -12821,7 +12821,7 @@
         <v>1.269999980926514</v>
       </c>
       <c r="I243" t="n">
-        <v>0.6800000071525574</v>
+        <v>0.5699999928474426</v>
       </c>
       <c r="J243" t="n">
         <v>0</v>
@@ -12833,10 +12833,10 @@
         <v>0.41</v>
       </c>
       <c r="M243" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.05</v>
       </c>
       <c r="N243" t="n">
-        <v>1.35</v>
+        <v>1.46</v>
       </c>
       <c r="O243" t="n">
         <v>3</v>
@@ -12872,7 +12872,7 @@
         <v>1.669999957084656</v>
       </c>
       <c r="I244" t="n">
-        <v>0.9300000071525574</v>
+        <v>0.8199999928474426</v>
       </c>
       <c r="J244" t="n">
         <v>0</v>
@@ -12884,10 +12884,10 @@
         <v>0.59</v>
       </c>
       <c r="M244" t="n">
-        <v>0.66</v>
+        <v>0.77</v>
       </c>
       <c r="N244" t="n">
-        <v>1.25</v>
+        <v>1.36</v>
       </c>
       <c r="O244" t="n">
         <v>2</v>
@@ -13076,7 +13076,7 @@
         <v>1.950000047683716</v>
       </c>
       <c r="I248" t="n">
-        <v>0.2099999934434891</v>
+        <v>0.1000000014901161</v>
       </c>
       <c r="J248" t="n">
         <v>0</v>
@@ -13088,10 +13088,10 @@
         <v>0.29</v>
       </c>
       <c r="M248" t="n">
-        <v>0.68</v>
+        <v>0.79</v>
       </c>
       <c r="N248" t="n">
-        <v>0.97</v>
+        <v>1.08</v>
       </c>
       <c r="O248" t="n">
         <v>3</v>
@@ -13178,7 +13178,7 @@
         <v>0.7900000214576721</v>
       </c>
       <c r="I250" t="n">
-        <v>0.8799999952316284</v>
+        <v>0.7699999809265137</v>
       </c>
       <c r="J250" t="n">
         <v>0</v>
@@ -13190,10 +13190,10 @@
         <v>0.23</v>
       </c>
       <c r="M250" t="n">
-        <v>0.91</v>
+        <v>1.02</v>
       </c>
       <c r="N250" t="n">
-        <v>1.14</v>
+        <v>1.25</v>
       </c>
       <c r="O250" t="n">
         <v>4</v>
@@ -13277,7 +13277,7 @@
         <v>0.705116610974073</v>
       </c>
       <c r="H252" t="n">
-        <v>1.129999995231628</v>
+        <v>1.019999980926514</v>
       </c>
       <c r="I252" t="n">
         <v>0.6399999856948853</v>
@@ -13289,13 +13289,13 @@
         <v>0</v>
       </c>
       <c r="L252" t="n">
-        <v>1.39</v>
+        <v>1.5</v>
       </c>
       <c r="M252" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="N252" t="n">
-        <v>1.46</v>
+        <v>1.57</v>
       </c>
       <c r="O252" t="n">
         <v>3</v>
@@ -13736,7 +13736,7 @@
         <v>0.5999353146180491</v>
       </c>
       <c r="H261" t="n">
-        <v>0.9200000166893005</v>
+        <v>0.8100000023841858</v>
       </c>
       <c r="I261" t="n">
         <v>0.6899999976158142</v>
@@ -13748,13 +13748,13 @@
         <v>0</v>
       </c>
       <c r="L261" t="n">
-        <v>0.62</v>
+        <v>0.73</v>
       </c>
       <c r="M261" t="n">
         <v>0.09</v>
       </c>
       <c r="N261" t="n">
-        <v>0.7</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="O261" t="n">
         <v>1</v>
@@ -13940,7 +13940,7 @@
         <v>0.208856437355279</v>
       </c>
       <c r="H265" t="n">
-        <v>1.210000038146973</v>
+        <v>1.100000023841858</v>
       </c>
       <c r="I265" t="n">
         <v>0.3300000131130219</v>
@@ -13952,13 +13952,13 @@
         <v>0</v>
       </c>
       <c r="L265" t="n">
-        <v>0.4</v>
+        <v>0.51</v>
       </c>
       <c r="M265" t="n">
         <v>0.12</v>
       </c>
       <c r="N265" t="n">
-        <v>0.52</v>
+        <v>0.63</v>
       </c>
       <c r="O265" t="n">
         <v>2</v>
@@ -14246,7 +14246,7 @@
         <v>0.733843019232151</v>
       </c>
       <c r="H271" t="n">
-        <v>0.8299999833106995</v>
+        <v>0.7200000286102295</v>
       </c>
       <c r="I271" t="n">
         <v>0.8999999761581421</v>
@@ -14258,13 +14258,13 @@
         <v>0</v>
       </c>
       <c r="L271" t="n">
-        <v>0.74</v>
+        <v>0.86</v>
       </c>
       <c r="M271" t="n">
         <v>0.16</v>
       </c>
       <c r="N271" t="n">
-        <v>0.91</v>
+        <v>1.02</v>
       </c>
       <c r="O271" t="n">
         <v>3</v>

</xml_diff>